<commit_message>
base de datos actualizada
</commit_message>
<xml_diff>
--- a/Base_De_Datos.xlsx
+++ b/Base_De_Datos.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\manuel\Desktop\uca\5\SIE\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\manue\Desktop\cosas-cosotas\5\SIE\SIE-Grupo-APPLE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FAFEA200-3835-4755-86B6-4C98F99F8321}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F56DCD3-52C0-45F2-A1E2-F64E164C5750}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{89460A5D-6D94-44C2-BF87-60F6987698AF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{89460A5D-6D94-44C2-BF87-60F6987698AF}"/>
   </bookViews>
   <sheets>
     <sheet name="Municipios" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="98">
   <si>
     <t>Municipio</t>
   </si>
@@ -52,9 +52,6 @@
     <t>Torre Alháquime</t>
   </si>
   <si>
-    <t>Zahara</t>
-  </si>
-  <si>
     <t>Algar</t>
   </si>
   <si>
@@ -157,32 +154,191 @@
     <t>Cargo</t>
   </si>
   <si>
-    <t>Agustín</t>
-  </si>
-  <si>
-    <t>Antonio</t>
-  </si>
-  <si>
-    <t>Jesús</t>
-  </si>
-  <si>
-    <t>Jose</t>
-  </si>
-  <si>
-    <t>Andrés</t>
-  </si>
-  <si>
-    <t>Lidia</t>
-  </si>
-  <si>
-    <t>Ana</t>
+    <t>Algeciras</t>
+  </si>
+  <si>
+    <t>Arcos de la Frontera</t>
+  </si>
+  <si>
+    <t>Barbate</t>
+  </si>
+  <si>
+    <t>Cádiz</t>
+  </si>
+  <si>
+    <t>Chiclana de la Frontera</t>
+  </si>
+  <si>
+    <t>Conil de la Frontera</t>
+  </si>
+  <si>
+    <t>El Puerto de Santa María</t>
+  </si>
+  <si>
+    <t>Jerez de la Frontera</t>
+  </si>
+  <si>
+    <t>La Línea de la Concepción</t>
+  </si>
+  <si>
+    <t>Los Barrios</t>
+  </si>
+  <si>
+    <t>Puerto Real</t>
+  </si>
+  <si>
+    <t>Rota</t>
+  </si>
+  <si>
+    <t>San Fernando</t>
+  </si>
+  <si>
+    <t>San Roque</t>
+  </si>
+  <si>
+    <t>Sanlúcar de Barrameda</t>
+  </si>
+  <si>
+    <t>Zahara de la Sierra</t>
+  </si>
+  <si>
+    <t>Mancomunidad de la Bahía de Cádiz</t>
+  </si>
+  <si>
+    <t>Mancomunidad de la Janda</t>
+  </si>
+  <si>
+    <t>Mancomunidad del Campo de Gibraltar</t>
+  </si>
+  <si>
+    <t>Mancounidad de la sierra de Cádiz</t>
+  </si>
+  <si>
+    <t>Zahara de los Atunes</t>
+  </si>
+  <si>
+    <t>Guadalcacín</t>
+  </si>
+  <si>
+    <t>La Barca de la Florida</t>
+  </si>
+  <si>
+    <t>El Torno</t>
+  </si>
+  <si>
+    <t>Nueva Jarilla</t>
+  </si>
+  <si>
+    <t>San Isidro del Guadalete</t>
+  </si>
+  <si>
+    <t>Estella del Marqués</t>
+  </si>
+  <si>
+    <t>Torrecera</t>
+  </si>
+  <si>
+    <t>Facinas</t>
+  </si>
+  <si>
+    <t>Tahivilla</t>
+  </si>
+  <si>
+    <t>D. Mario Martín Ojeda</t>
+  </si>
+  <si>
+    <t>D. Óscar Palma Toledo</t>
+  </si>
+  <si>
+    <t>Dª. Rosa Alonso Rodríguez</t>
+  </si>
+  <si>
+    <t>Dª. Rocío Romero Sánchez</t>
+  </si>
+  <si>
+    <t>D. Rogelio Navarrete Manchado</t>
+  </si>
+  <si>
+    <t>D. Raúl Espinar Torres</t>
+  </si>
+  <si>
+    <t>Dª. María Dulce García Durán</t>
+  </si>
+  <si>
+    <t>D. Guillermo Muñoz-Delgado Serrano</t>
+  </si>
+  <si>
+    <t>Dª. Belén María Robles Brioso</t>
+  </si>
+  <si>
+    <t>Dª. Vanessa Braza Blanco</t>
+  </si>
+  <si>
+    <t>Dª. Rocío Ana González Iborra</t>
+  </si>
+  <si>
+    <t>D. Jorge Grimaldi Torres</t>
+  </si>
+  <si>
+    <t>D. José Manuel Pérez Alcaraz</t>
+  </si>
+  <si>
+    <t>D. Javier Clavijo González</t>
+  </si>
+  <si>
+    <t>D. Fernando Díaz Ortega</t>
+  </si>
+  <si>
+    <t>Dª. María Patrocinio Gómez-Collantes</t>
+  </si>
+  <si>
+    <t>Dª. María Victoria Mayorga Rubio</t>
+  </si>
+  <si>
+    <t>Dª. Elena Vidal Perez</t>
+  </si>
+  <si>
+    <t>Dª. Elena Zambrano Romero</t>
+  </si>
+  <si>
+    <t>Dª. Isabel Sánchez Gil</t>
+  </si>
+  <si>
+    <t>Dª. Agueda Leal Quiñones</t>
+  </si>
+  <si>
+    <t>D. Agustín Martinez López</t>
+  </si>
+  <si>
+    <t>D. Antonio Jesús Sánchez Guirado</t>
+  </si>
+  <si>
+    <t>D. Jose María Dianez Sánchez</t>
+  </si>
+  <si>
+    <t>D. Jose Eduardo Galindo Merchán</t>
+  </si>
+  <si>
+    <t>D. Francisco José Martínez Alba</t>
+  </si>
+  <si>
+    <t>Dª. Mª José Álvarez Luna</t>
+  </si>
+  <si>
+    <t>Dª. María Fley Báez</t>
+  </si>
+  <si>
+    <t>Dª. Mª Jesús Rodríguez Fernández</t>
+  </si>
+  <si>
+    <t>D. Carlos García Rodríguez</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -190,16 +346,40 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5F7FA"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -207,12 +387,39 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -547,266 +754,528 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3606FAFD-1884-47F2-8486-B1950726AF05}">
-  <dimension ref="A1:A31"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:A60"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="30.85546875" customWidth="1"/>
+    <col min="1" max="1" width="30.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A40" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A41" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A42" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A43" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+    <row r="44" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A44" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A45" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A46" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A47" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A48" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A49" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A50" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A51" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A52" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A53" s="3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A54" s="3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A55" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A56" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A57" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A58" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>28</v>
+    <row r="59" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A59" s="3" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A60" s="3" t="s">
+        <v>67</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{473D6359-92CE-479F-9B62-92C1E4CE4353}">
-  <dimension ref="A1:A8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:A31"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.140625" customWidth="1"/>
+    <col min="1" max="1" width="29.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>45</v>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="4" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="4" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="4" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="4" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="4" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="4" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="4" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="4" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="4" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="4" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="4" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="4" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="4" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="4" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="4" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="4" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="4" t="s">
+        <v>97</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{195EBCBB-C110-4D7C-9373-C6B300948B3C}">
   <dimension ref="A1:A7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.28515625" customWidth="1"/>
+    <col min="1" max="1" width="24.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>36</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>